<commit_message>
update data package at: 2026-08-28T08:05:28
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E295"/>
+  <dimension ref="A1:E297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6531,11 +6531,11 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>5764</v>
+        <v>613</v>
       </c>
     </row>
     <row r="267">
@@ -6554,11 +6554,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>4671</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="268">
@@ -6577,11 +6577,11 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>1358</v>
+        <v>4354</v>
       </c>
     </row>
     <row r="269">
@@ -6600,11 +6600,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>850</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="270">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -6623,11 +6623,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>2</v>
+        <v>844</v>
       </c>
     </row>
     <row r="271">
@@ -6636,21 +6636,21 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>61</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="272">
@@ -6669,11 +6669,11 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
     </row>
     <row r="273">
@@ -6692,11 +6692,11 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>147</v>
+        <v>61</v>
       </c>
     </row>
     <row r="274">
@@ -6715,11 +6715,11 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="275">
@@ -6738,11 +6738,11 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>1</v>
+        <v>147</v>
       </c>
     </row>
     <row r="276">
@@ -6756,16 +6756,16 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>283</v>
+        <v>3</v>
       </c>
     </row>
     <row r="277">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -6784,11 +6784,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="278">
@@ -6797,21 +6797,21 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>4</v>
+        <v>283</v>
       </c>
     </row>
     <row r="279">
@@ -6830,11 +6830,11 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>513</v>
+        <v>3</v>
       </c>
     </row>
     <row r="280">
@@ -6853,11 +6853,11 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>863</v>
+        <v>4</v>
       </c>
     </row>
     <row r="281">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -6876,11 +6876,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>149</v>
+        <v>513</v>
       </c>
     </row>
     <row r="282">
@@ -6889,7 +6889,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -6899,11 +6899,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>38</v>
+        <v>863</v>
       </c>
     </row>
     <row r="283">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6922,11 +6922,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="284">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6945,11 +6945,11 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>158</v>
+        <v>38</v>
       </c>
     </row>
     <row r="285">
@@ -6968,11 +6968,11 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
     </row>
     <row r="286">
@@ -6991,11 +6991,11 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>38</v>
+        <v>158</v>
       </c>
     </row>
     <row r="287">
@@ -7014,11 +7014,11 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>1</v>
+        <v>56</v>
       </c>
     </row>
     <row r="288">
@@ -7032,16 +7032,16 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>273</v>
+        <v>38</v>
       </c>
     </row>
     <row r="289">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7060,7 +7060,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E289" t="n">
@@ -7073,21 +7073,21 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>24</v>
+        <v>273</v>
       </c>
     </row>
     <row r="291">
@@ -7106,11 +7106,11 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="292">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="293">
@@ -7152,11 +7152,11 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
     <row r="294">
@@ -7170,12 +7170,12 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E294" t="n">
@@ -7188,20 +7188,66 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
           <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
-      <c r="C295" t="inlineStr">
+      <c r="C297" t="inlineStr">
         <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr">
+      <c r="D297" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E295" t="n">
+      <c r="E297" t="n">
         <v>1703</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update data package at: 2026-08-31T08:59:01
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E297"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4304,7 +4304,7 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>38121</v>
+        <v>38749</v>
       </c>
     </row>
     <row r="170">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="292">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -7133,7 +7133,7 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="293">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7156,7 +7156,7 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="294">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -7179,7 +7179,7 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
     </row>
     <row r="295">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7198,11 +7198,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>40</v>
+        <v>282</v>
       </c>
     </row>
     <row r="296">
@@ -7211,21 +7211,21 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>32</v>
+        <v>205</v>
       </c>
     </row>
     <row r="297">
@@ -7234,21 +7234,343 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
+          <t>2151 - FHA</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2421 - IDENE</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
           <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
-      <c r="C297" t="inlineStr">
+      <c r="C304" t="inlineStr">
         <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr">
+      <c r="D304" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E297" t="n">
+      <c r="E304" t="n">
         <v>1703</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>175450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update data package at: 2026-09-01T12:46:25
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E311"/>
+  <dimension ref="A1:E312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3844,7 +3844,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="151">
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>455</v>
+        <v>313</v>
       </c>
     </row>
     <row r="152">
@@ -3904,16 +3904,16 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>1529</v>
+        <v>133</v>
       </c>
     </row>
     <row r="153">
@@ -3922,21 +3922,21 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>1</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="154">
@@ -3955,11 +3955,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -3978,11 +3978,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="156">
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>99</v>
+        <v>43</v>
       </c>
     </row>
     <row r="157">
@@ -4019,16 +4019,16 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>51</v>
+        <v>99</v>
       </c>
     </row>
     <row r="158">
@@ -4037,21 +4037,21 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
     </row>
     <row r="159">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4093,11 +4093,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="161">
@@ -4116,11 +4116,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>258</v>
+        <v>3</v>
       </c>
     </row>
     <row r="162">
@@ -4139,11 +4139,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>1</v>
+        <v>258</v>
       </c>
     </row>
     <row r="163">
@@ -4162,11 +4162,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>243</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -4185,11 +4185,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>2855</v>
+        <v>243</v>
       </c>
     </row>
     <row r="165">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>1828</v>
+        <v>2855</v>
       </c>
     </row>
     <row r="166">
@@ -4231,11 +4231,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>3483</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="167">
@@ -4254,11 +4254,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>34165</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="168">
@@ -4272,16 +4272,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>874</v>
+        <v>34165</v>
       </c>
     </row>
     <row r="169">
@@ -4300,11 +4300,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>38749</v>
+        <v>874</v>
       </c>
     </row>
     <row r="170">
@@ -4313,21 +4313,21 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>3</v>
+        <v>38749</v>
       </c>
     </row>
     <row r="171">
@@ -4346,11 +4346,11 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172">
@@ -4369,11 +4369,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
     </row>
     <row r="173">
@@ -4392,11 +4392,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>13</v>
+        <v>83</v>
       </c>
     </row>
     <row r="174">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="175">
@@ -4428,21 +4428,21 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>151</v>
+        <v>22</v>
       </c>
     </row>
     <row r="176">
@@ -4451,21 +4451,21 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="177">
@@ -4484,11 +4484,11 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
@@ -4507,11 +4507,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="179">
@@ -4530,11 +4530,11 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
     </row>
     <row r="180">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="181">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4576,11 +4576,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>135</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -4589,21 +4589,21 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>65</v>
+        <v>135</v>
       </c>
     </row>
     <row r="183">
@@ -4612,21 +4612,21 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>2</v>
+        <v>65</v>
       </c>
     </row>
     <row r="184">
@@ -4645,11 +4645,11 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="185">
@@ -4668,11 +4668,11 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>794</v>
+        <v>22</v>
       </c>
     </row>
     <row r="186">
@@ -4691,11 +4691,11 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>5154</v>
+        <v>794</v>
       </c>
     </row>
     <row r="187">
@@ -4709,16 +4709,16 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>3190</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="188">
@@ -4727,21 +4727,21 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>2</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="189">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="190">
@@ -4778,16 +4778,16 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="191">
@@ -4801,16 +4801,16 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="192">
@@ -4819,21 +4819,21 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="193">
@@ -4852,11 +4852,11 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>769</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194">
@@ -4875,11 +4875,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>1440</v>
+        <v>769</v>
       </c>
     </row>
     <row r="195">
@@ -4898,11 +4898,11 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>533</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="196">
@@ -4916,16 +4916,16 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>4251</v>
+        <v>533</v>
       </c>
     </row>
     <row r="197">
@@ -4934,21 +4934,21 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>5</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="198">
@@ -4967,11 +4967,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>117</v>
+        <v>5</v>
       </c>
     </row>
     <row r="199">
@@ -4990,11 +4990,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>17</v>
+        <v>117</v>
       </c>
     </row>
     <row r="200">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -5036,11 +5036,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="202">
@@ -5054,16 +5054,16 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>317</v>
+        <v>31</v>
       </c>
     </row>
     <row r="203">
@@ -5072,21 +5072,21 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>43</v>
+        <v>317</v>
       </c>
     </row>
     <row r="204">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>295</v>
+        <v>43</v>
       </c>
     </row>
     <row r="205">
@@ -5128,11 +5128,11 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>120</v>
+        <v>295</v>
       </c>
     </row>
     <row r="206">
@@ -5151,11 +5151,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>175</v>
+        <v>120</v>
       </c>
     </row>
     <row r="207">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5174,11 +5174,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>7</v>
+        <v>175</v>
       </c>
     </row>
     <row r="208">
@@ -5197,11 +5197,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="209">
@@ -5220,11 +5220,11 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>121</v>
+        <v>45</v>
       </c>
     </row>
     <row r="210">
@@ -5243,11 +5243,11 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>85</v>
+        <v>121</v>
       </c>
     </row>
     <row r="211">
@@ -5261,16 +5261,16 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="212">
@@ -5279,21 +5279,21 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>3</v>
+        <v>71</v>
       </c>
     </row>
     <row r="213">
@@ -5312,11 +5312,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214">
@@ -5335,11 +5335,11 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>94</v>
+        <v>27</v>
       </c>
     </row>
     <row r="215">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>25</v>
+        <v>94</v>
       </c>
     </row>
     <row r="216">
@@ -5381,11 +5381,11 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="217">
@@ -5404,11 +5404,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="218">
@@ -5422,16 +5422,16 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E218" t="n">
-        <v>124</v>
+        <v>36</v>
       </c>
     </row>
     <row r="219">
@@ -5440,21 +5440,21 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2281 - UTRAMIG</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>10</v>
+        <v>124</v>
       </c>
     </row>
     <row r="220">
@@ -5473,11 +5473,11 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2281 - UTRAMIG</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5496,11 +5496,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="222">
@@ -5519,11 +5519,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="223">
@@ -5542,11 +5542,11 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>898</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224">
@@ -5565,11 +5565,11 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>11</v>
+        <v>898</v>
       </c>
     </row>
     <row r="225">
@@ -5588,11 +5588,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>343</v>
+        <v>11</v>
       </c>
     </row>
     <row r="226">
@@ -5606,16 +5606,16 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E226" t="n">
-        <v>595</v>
+        <v>343</v>
       </c>
     </row>
     <row r="227">
@@ -5629,16 +5629,16 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E227" t="n">
-        <v>48</v>
+        <v>595</v>
       </c>
     </row>
     <row r="228">
@@ -5647,21 +5647,21 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E228" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="229">
@@ -5680,11 +5680,11 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E229" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230">
@@ -5703,11 +5703,11 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E230" t="n">
-        <v>224</v>
+        <v>26</v>
       </c>
     </row>
     <row r="231">
@@ -5726,11 +5726,11 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E231" t="n">
-        <v>282</v>
+        <v>224</v>
       </c>
     </row>
     <row r="232">
@@ -5749,11 +5749,11 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>183</v>
+        <v>282</v>
       </c>
     </row>
     <row r="233">
@@ -5767,16 +5767,16 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>276</v>
+        <v>183</v>
       </c>
     </row>
     <row r="234">
@@ -5785,21 +5785,21 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>8</v>
+        <v>276</v>
       </c>
     </row>
     <row r="235">
@@ -5818,11 +5818,11 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>946</v>
+        <v>8</v>
       </c>
     </row>
     <row r="236">
@@ -5841,11 +5841,11 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>1350</v>
+        <v>946</v>
       </c>
     </row>
     <row r="237">
@@ -5864,11 +5864,11 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>1351</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="238">
@@ -5887,11 +5887,11 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>1138</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="239">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5910,11 +5910,11 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>1</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="240">
@@ -5923,21 +5923,21 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>829</v>
+        <v>1</v>
       </c>
     </row>
     <row r="241">
@@ -5946,21 +5946,21 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>33</v>
+        <v>829</v>
       </c>
     </row>
     <row r="242">
@@ -5979,11 +5979,11 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>75</v>
+        <v>33</v>
       </c>
     </row>
     <row r="243">
@@ -6002,11 +6002,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>364</v>
+        <v>75</v>
       </c>
     </row>
     <row r="244">
@@ -6025,11 +6025,11 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>534</v>
+        <v>364</v>
       </c>
     </row>
     <row r="245">
@@ -6048,11 +6048,11 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>2500</v>
+        <v>534</v>
       </c>
     </row>
     <row r="246">
@@ -6071,11 +6071,11 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>24</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="247">
@@ -6094,11 +6094,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="248">
@@ -6112,16 +6112,16 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>1251</v>
+        <v>77</v>
       </c>
     </row>
     <row r="249">
@@ -6130,21 +6130,21 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>2</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="250">
@@ -6163,11 +6163,11 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>91</v>
+        <v>2</v>
       </c>
     </row>
     <row r="251">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>2</v>
+        <v>91</v>
       </c>
     </row>
     <row r="252">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2431 - AGÊNCIA RMBH</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -6209,11 +6209,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="253">
@@ -6232,11 +6232,11 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="254">
@@ -6255,11 +6255,11 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="255">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2431 - AGÊNCIA RMBH</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6278,11 +6278,11 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="256">
@@ -6301,11 +6301,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
     </row>
     <row r="257">
@@ -6324,11 +6324,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>131</v>
+        <v>53</v>
       </c>
     </row>
     <row r="258">
@@ -6342,16 +6342,16 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>2</v>
+        <v>131</v>
       </c>
     </row>
     <row r="259">
@@ -6365,16 +6365,16 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>398</v>
+        <v>2</v>
       </c>
     </row>
     <row r="260">
@@ -6383,21 +6383,21 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>1</v>
+        <v>398</v>
       </c>
     </row>
     <row r="261">
@@ -6416,11 +6416,11 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="262">
@@ -6439,11 +6439,11 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="263">
@@ -6462,11 +6462,11 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>286</v>
+        <v>54</v>
       </c>
     </row>
     <row r="264">
@@ -6480,16 +6480,16 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>95</v>
+        <v>286</v>
       </c>
     </row>
     <row r="265">
@@ -6498,21 +6498,21 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
     </row>
     <row r="266">
@@ -6531,11 +6531,11 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>613</v>
+        <v>2</v>
       </c>
     </row>
     <row r="267">
@@ -6554,11 +6554,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>5712</v>
+        <v>613</v>
       </c>
     </row>
     <row r="268">
@@ -6577,11 +6577,11 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>4354</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="269">
@@ -6600,11 +6600,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>1146</v>
+        <v>4354</v>
       </c>
     </row>
     <row r="270">
@@ -6623,11 +6623,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>844</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="271">
@@ -6641,16 +6641,16 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>4085</v>
+        <v>844</v>
       </c>
     </row>
     <row r="272">
@@ -6659,21 +6659,21 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>2</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="273">
@@ -6692,11 +6692,11 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
     </row>
     <row r="274">
@@ -6715,11 +6715,11 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
     </row>
     <row r="275">
@@ -6738,11 +6738,11 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>147</v>
+        <v>36</v>
       </c>
     </row>
     <row r="276">
@@ -6761,11 +6761,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>3</v>
+        <v>147</v>
       </c>
     </row>
     <row r="277">
@@ -6784,11 +6784,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="278">
@@ -6802,16 +6802,16 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>283</v>
+        <v>1</v>
       </c>
     </row>
     <row r="279">
@@ -6820,21 +6820,21 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>3</v>
+        <v>283</v>
       </c>
     </row>
     <row r="280">
@@ -6853,11 +6853,11 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="281">
@@ -6876,11 +6876,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>513</v>
+        <v>4</v>
       </c>
     </row>
     <row r="282">
@@ -6899,11 +6899,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>863</v>
+        <v>513</v>
       </c>
     </row>
     <row r="283">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6926,7 +6926,7 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>149</v>
+        <v>863</v>
       </c>
     </row>
     <row r="284">
@@ -6945,11 +6945,11 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>38</v>
+        <v>149</v>
       </c>
     </row>
     <row r="285">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -6968,11 +6968,11 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
     </row>
     <row r="286">
@@ -6991,11 +6991,11 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>158</v>
+        <v>4</v>
       </c>
     </row>
     <row r="287">
@@ -7014,11 +7014,11 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>56</v>
+        <v>158</v>
       </c>
     </row>
     <row r="288">
@@ -7037,11 +7037,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="289">
@@ -7060,11 +7060,11 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="290">
@@ -7078,16 +7078,16 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>273</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
@@ -7096,21 +7096,21 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>7</v>
+        <v>273</v>
       </c>
     </row>
     <row r="292">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="293">
@@ -7152,11 +7152,11 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="294">
@@ -7175,11 +7175,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="295">
@@ -7198,11 +7198,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>282</v>
+        <v>48</v>
       </c>
     </row>
     <row r="296">
@@ -7221,11 +7221,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>205</v>
+        <v>282</v>
       </c>
     </row>
     <row r="297">
@@ -7239,16 +7239,16 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>53</v>
+        <v>205</v>
       </c>
     </row>
     <row r="298">
@@ -7257,21 +7257,21 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
     </row>
     <row r="299">
@@ -7290,11 +7290,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="300">
@@ -7313,11 +7313,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="301">
@@ -7336,11 +7336,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="302">
@@ -7359,11 +7359,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="303">
@@ -7377,16 +7377,16 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="304">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7409,7 +7409,7 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>1703</v>
+        <v>32</v>
       </c>
     </row>
     <row r="305">
@@ -7418,21 +7418,21 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>6</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="306">
@@ -7451,11 +7451,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>4125</v>
+        <v>6</v>
       </c>
     </row>
     <row r="307">
@@ -7474,11 +7474,11 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>21486</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="308">
@@ -7497,11 +7497,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>14673</v>
+        <v>21486</v>
       </c>
     </row>
     <row r="309">
@@ -7520,11 +7520,11 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>155811</v>
+        <v>14673</v>
       </c>
     </row>
     <row r="310">
@@ -7543,11 +7543,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>39906</v>
+        <v>155811</v>
       </c>
     </row>
     <row r="311">
@@ -7561,15 +7561,38 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr">
+      <c r="D312" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E311" t="n">
+      <c r="E312" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update data package at: 2026-09-02T08:44:00
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E312"/>
+  <dimension ref="A1:E316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7317,7 +7317,7 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="301">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7336,11 +7336,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="302">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7359,11 +7359,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="303">
@@ -7382,11 +7382,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="304">
@@ -7400,16 +7400,16 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="305">
@@ -7418,21 +7418,21 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>1703</v>
+        <v>16</v>
       </c>
     </row>
     <row r="306">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7451,11 +7451,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="307">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7474,11 +7474,11 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>4125</v>
+        <v>40</v>
       </c>
     </row>
     <row r="308">
@@ -7487,21 +7487,21 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>21486</v>
+        <v>32</v>
       </c>
     </row>
     <row r="309">
@@ -7510,21 +7510,21 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>14673</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="310">
@@ -7543,11 +7543,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>155811</v>
+        <v>6</v>
       </c>
     </row>
     <row r="311">
@@ -7566,11 +7566,11 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>39906</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="312">
@@ -7584,15 +7584,107 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr">
+      <c r="D316" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E312" t="n">
+      <c r="E316" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update data package at: 2026-09-03T08:36:59
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E316"/>
+  <dimension ref="A1:E323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="145">
@@ -3752,7 +3752,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="146">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="147">
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>1688</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="148">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="149">
@@ -3830,21 +3830,21 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2351 - UEMG</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>11</v>
+        <v>505</v>
       </c>
     </row>
     <row r="150">
@@ -3863,11 +3863,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>663</v>
+        <v>11</v>
       </c>
     </row>
     <row r="151">
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>313</v>
+        <v>663</v>
       </c>
     </row>
     <row r="152">
@@ -3909,11 +3909,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>133</v>
+        <v>313</v>
       </c>
     </row>
     <row r="153">
@@ -3927,16 +3927,16 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>1529</v>
+        <v>133</v>
       </c>
     </row>
     <row r="154">
@@ -3945,21 +3945,21 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>1</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="155">
@@ -3978,11 +3978,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="157">
@@ -4024,11 +4024,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>99</v>
+        <v>43</v>
       </c>
     </row>
     <row r="158">
@@ -4042,16 +4042,16 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>51</v>
+        <v>99</v>
       </c>
     </row>
     <row r="159">
@@ -4060,21 +4060,21 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
     </row>
     <row r="160">
@@ -4093,11 +4093,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4116,11 +4116,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="162">
@@ -4139,11 +4139,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>258</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163">
@@ -4162,11 +4162,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>1</v>
+        <v>258</v>
       </c>
     </row>
     <row r="164">
@@ -4185,11 +4185,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>243</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>2855</v>
+        <v>243</v>
       </c>
     </row>
     <row r="166">
@@ -4231,11 +4231,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>1828</v>
+        <v>2855</v>
       </c>
     </row>
     <row r="167">
@@ -4254,11 +4254,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>3483</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="168">
@@ -4277,11 +4277,11 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>34165</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="169">
@@ -4295,16 +4295,16 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>874</v>
+        <v>34165</v>
       </c>
     </row>
     <row r="170">
@@ -4323,11 +4323,11 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>38749</v>
+        <v>874</v>
       </c>
     </row>
     <row r="171">
@@ -4336,21 +4336,21 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>3</v>
+        <v>38749</v>
       </c>
     </row>
     <row r="172">
@@ -4369,11 +4369,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173">
@@ -4392,11 +4392,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
     </row>
     <row r="174">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>13</v>
+        <v>83</v>
       </c>
     </row>
     <row r="175">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4438,11 +4438,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="176">
@@ -4451,21 +4451,21 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>151</v>
+        <v>22</v>
       </c>
     </row>
     <row r="177">
@@ -4474,21 +4474,21 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="178">
@@ -4507,11 +4507,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179">
@@ -4530,11 +4530,11 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="180">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
     </row>
     <row r="181">
@@ -4576,11 +4576,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="182">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4599,11 +4599,11 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>135</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -4612,21 +4612,21 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>65</v>
+        <v>135</v>
       </c>
     </row>
     <row r="184">
@@ -4635,21 +4635,21 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>2</v>
+        <v>65</v>
       </c>
     </row>
     <row r="185">
@@ -4668,11 +4668,11 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="186">
@@ -4691,11 +4691,11 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>794</v>
+        <v>22</v>
       </c>
     </row>
     <row r="187">
@@ -4714,11 +4714,11 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>5154</v>
+        <v>794</v>
       </c>
     </row>
     <row r="188">
@@ -4732,16 +4732,16 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>3190</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="189">
@@ -4750,21 +4750,21 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>2</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="190">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191">
@@ -4801,16 +4801,16 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="192">
@@ -4824,16 +4824,16 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193">
@@ -4842,21 +4842,21 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="194">
@@ -4875,11 +4875,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>769</v>
+        <v>5</v>
       </c>
     </row>
     <row r="195">
@@ -4898,11 +4898,11 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>1440</v>
+        <v>769</v>
       </c>
     </row>
     <row r="196">
@@ -4921,11 +4921,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>533</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="197">
@@ -4939,16 +4939,16 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>4251</v>
+        <v>533</v>
       </c>
     </row>
     <row r="198">
@@ -4957,21 +4957,21 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>5</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="199">
@@ -4990,11 +4990,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>117</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200">
@@ -5013,11 +5013,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>17</v>
+        <v>117</v>
       </c>
     </row>
     <row r="201">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -5059,11 +5059,11 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="203">
@@ -5077,16 +5077,16 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>317</v>
+        <v>31</v>
       </c>
     </row>
     <row r="204">
@@ -5095,21 +5095,21 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>43</v>
+        <v>317</v>
       </c>
     </row>
     <row r="205">
@@ -5128,11 +5128,11 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>295</v>
+        <v>43</v>
       </c>
     </row>
     <row r="206">
@@ -5151,11 +5151,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>120</v>
+        <v>295</v>
       </c>
     </row>
     <row r="207">
@@ -5174,11 +5174,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>175</v>
+        <v>120</v>
       </c>
     </row>
     <row r="208">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5197,11 +5197,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>7</v>
+        <v>175</v>
       </c>
     </row>
     <row r="209">
@@ -5220,11 +5220,11 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="210">
@@ -5243,11 +5243,11 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>121</v>
+        <v>45</v>
       </c>
     </row>
     <row r="211">
@@ -5266,11 +5266,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>85</v>
+        <v>121</v>
       </c>
     </row>
     <row r="212">
@@ -5284,16 +5284,16 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="213">
@@ -5302,21 +5302,21 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>3</v>
+        <v>71</v>
       </c>
     </row>
     <row r="214">
@@ -5335,11 +5335,11 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>94</v>
+        <v>27</v>
       </c>
     </row>
     <row r="216">
@@ -5381,11 +5381,11 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>25</v>
+        <v>94</v>
       </c>
     </row>
     <row r="217">
@@ -5404,11 +5404,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="218">
@@ -5427,11 +5427,11 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E218" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="219">
@@ -5445,16 +5445,16 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>124</v>
+        <v>36</v>
       </c>
     </row>
     <row r="220">
@@ -5463,21 +5463,21 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2281 - UTRAMIG</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>10</v>
+        <v>124</v>
       </c>
     </row>
     <row r="221">
@@ -5496,11 +5496,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2281 - UTRAMIG</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5519,11 +5519,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="223">
@@ -5542,11 +5542,11 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224">
@@ -5565,11 +5565,11 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>898</v>
+        <v>38</v>
       </c>
     </row>
     <row r="225">
@@ -5588,11 +5588,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>11</v>
+        <v>898</v>
       </c>
     </row>
     <row r="226">
@@ -5611,11 +5611,11 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E226" t="n">
-        <v>343</v>
+        <v>11</v>
       </c>
     </row>
     <row r="227">
@@ -5629,16 +5629,16 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E227" t="n">
-        <v>595</v>
+        <v>343</v>
       </c>
     </row>
     <row r="228">
@@ -5652,16 +5652,16 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E228" t="n">
-        <v>48</v>
+        <v>595</v>
       </c>
     </row>
     <row r="229">
@@ -5670,21 +5670,21 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E229" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="230">
@@ -5703,11 +5703,11 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E230" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231">
@@ -5726,11 +5726,11 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E231" t="n">
-        <v>224</v>
+        <v>26</v>
       </c>
     </row>
     <row r="232">
@@ -5749,11 +5749,11 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>282</v>
+        <v>224</v>
       </c>
     </row>
     <row r="233">
@@ -5772,11 +5772,11 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>183</v>
+        <v>282</v>
       </c>
     </row>
     <row r="234">
@@ -5790,16 +5790,16 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>276</v>
+        <v>183</v>
       </c>
     </row>
     <row r="235">
@@ -5808,21 +5808,21 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>8</v>
+        <v>276</v>
       </c>
     </row>
     <row r="236">
@@ -5841,11 +5841,11 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>946</v>
+        <v>8</v>
       </c>
     </row>
     <row r="237">
@@ -5864,11 +5864,11 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>1350</v>
+        <v>946</v>
       </c>
     </row>
     <row r="238">
@@ -5887,11 +5887,11 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>1351</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="239">
@@ -5910,11 +5910,11 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>1138</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="240">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>1</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="241">
@@ -5946,21 +5946,21 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>829</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242">
@@ -5969,21 +5969,21 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>33</v>
+        <v>829</v>
       </c>
     </row>
     <row r="243">
@@ -6002,11 +6002,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>75</v>
+        <v>33</v>
       </c>
     </row>
     <row r="244">
@@ -6025,11 +6025,11 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>364</v>
+        <v>75</v>
       </c>
     </row>
     <row r="245">
@@ -6048,11 +6048,11 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>534</v>
+        <v>364</v>
       </c>
     </row>
     <row r="246">
@@ -6071,11 +6071,11 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>2500</v>
+        <v>534</v>
       </c>
     </row>
     <row r="247">
@@ -6094,11 +6094,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>24</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="248">
@@ -6117,11 +6117,11 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="249">
@@ -6135,16 +6135,16 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>1251</v>
+        <v>77</v>
       </c>
     </row>
     <row r="250">
@@ -6153,21 +6153,21 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>2</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="251">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>91</v>
+        <v>2</v>
       </c>
     </row>
     <row r="252">
@@ -6209,11 +6209,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>2</v>
+        <v>91</v>
       </c>
     </row>
     <row r="253">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2431 - AGÊNCIA RMBH</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -6232,11 +6232,11 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="254">
@@ -6255,11 +6255,11 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="255">
@@ -6278,11 +6278,11 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="256">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2431 - AGÊNCIA RMBH</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6301,11 +6301,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="257">
@@ -6324,11 +6324,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
     </row>
     <row r="258">
@@ -6347,11 +6347,11 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>131</v>
+        <v>53</v>
       </c>
     </row>
     <row r="259">
@@ -6365,16 +6365,16 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>2</v>
+        <v>131</v>
       </c>
     </row>
     <row r="260">
@@ -6388,16 +6388,16 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>398</v>
+        <v>2</v>
       </c>
     </row>
     <row r="261">
@@ -6406,21 +6406,21 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>1</v>
+        <v>398</v>
       </c>
     </row>
     <row r="262">
@@ -6439,11 +6439,11 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="263">
@@ -6462,11 +6462,11 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="264">
@@ -6485,11 +6485,11 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>286</v>
+        <v>54</v>
       </c>
     </row>
     <row r="265">
@@ -6503,16 +6503,16 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>95</v>
+        <v>286</v>
       </c>
     </row>
     <row r="266">
@@ -6521,21 +6521,21 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
     </row>
     <row r="267">
@@ -6554,11 +6554,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>613</v>
+        <v>2</v>
       </c>
     </row>
     <row r="268">
@@ -6577,11 +6577,11 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>5712</v>
+        <v>613</v>
       </c>
     </row>
     <row r="269">
@@ -6600,11 +6600,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>4354</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="270">
@@ -6623,11 +6623,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>1146</v>
+        <v>4354</v>
       </c>
     </row>
     <row r="271">
@@ -6646,11 +6646,11 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>844</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="272">
@@ -6664,16 +6664,16 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>4085</v>
+        <v>844</v>
       </c>
     </row>
     <row r="273">
@@ -6682,21 +6682,21 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>2</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="274">
@@ -6715,11 +6715,11 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
     </row>
     <row r="275">
@@ -6738,11 +6738,11 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
     </row>
     <row r="276">
@@ -6761,11 +6761,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>147</v>
+        <v>36</v>
       </c>
     </row>
     <row r="277">
@@ -6784,11 +6784,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>3</v>
+        <v>147</v>
       </c>
     </row>
     <row r="278">
@@ -6807,11 +6807,11 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="279">
@@ -6825,16 +6825,16 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>283</v>
+        <v>1</v>
       </c>
     </row>
     <row r="280">
@@ -6843,21 +6843,21 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>3</v>
+        <v>283</v>
       </c>
     </row>
     <row r="281">
@@ -6876,11 +6876,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="282">
@@ -6899,11 +6899,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>513</v>
+        <v>4</v>
       </c>
     </row>
     <row r="283">
@@ -6922,11 +6922,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>863</v>
+        <v>513</v>
       </c>
     </row>
     <row r="284">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6949,7 +6949,7 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>149</v>
+        <v>863</v>
       </c>
     </row>
     <row r="285">
@@ -6968,11 +6968,11 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>38</v>
+        <v>149</v>
       </c>
     </row>
     <row r="286">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -6991,11 +6991,11 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
     </row>
     <row r="287">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -7014,11 +7014,11 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>158</v>
+        <v>1</v>
       </c>
     </row>
     <row r="288">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7037,11 +7037,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>56</v>
+        <v>217</v>
       </c>
     </row>
     <row r="289">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7060,11 +7060,11 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>38</v>
+        <v>227</v>
       </c>
     </row>
     <row r="290">
@@ -7073,7 +7073,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="291">
@@ -7096,21 +7096,21 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>273</v>
+        <v>10</v>
       </c>
     </row>
     <row r="292">
@@ -7119,21 +7119,21 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>7</v>
+        <v>411</v>
       </c>
     </row>
     <row r="293">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7152,11 +7152,11 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="294">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -7175,11 +7175,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>22</v>
+        <v>158</v>
       </c>
     </row>
     <row r="295">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7198,11 +7198,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="296">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7221,11 +7221,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>282</v>
+        <v>38</v>
       </c>
     </row>
     <row r="297">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7244,11 +7244,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>205</v>
+        <v>1</v>
       </c>
     </row>
     <row r="298">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>53</v>
+        <v>273</v>
       </c>
     </row>
     <row r="299">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -7294,7 +7294,7 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="300">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7317,7 +7317,7 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="301">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7336,11 +7336,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="302">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7359,11 +7359,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="303">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7382,11 +7382,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>1</v>
+        <v>282</v>
       </c>
     </row>
     <row r="304">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7405,11 +7405,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>24</v>
+        <v>205</v>
       </c>
     </row>
     <row r="305">
@@ -7418,21 +7418,21 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>16</v>
+        <v>53</v>
       </c>
     </row>
     <row r="306">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7451,11 +7451,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7474,11 +7474,11 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="308">
@@ -7487,21 +7487,21 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="309">
@@ -7510,21 +7510,21 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>1703</v>
+        <v>17</v>
       </c>
     </row>
     <row r="310">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7547,7 +7547,7 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7570,7 +7570,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>4125</v>
+        <v>24</v>
       </c>
     </row>
     <row r="312">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -7593,7 +7593,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>21486</v>
+        <v>16</v>
       </c>
     </row>
     <row r="313">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7616,7 +7616,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>14673</v>
+        <v>32</v>
       </c>
     </row>
     <row r="314">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7635,11 +7635,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>155811</v>
+        <v>40</v>
       </c>
     </row>
     <row r="315">
@@ -7648,21 +7648,21 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>39906</v>
+        <v>32</v>
       </c>
     </row>
     <row r="316">
@@ -7671,20 +7671,181 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
+          <t>1941 - EGE-SEPLAG</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
           <t>1261 - SEE</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr">
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
         <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr">
+      <c r="D323" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E316" t="n">
+      <c r="E323" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update data package at: 2026-09-08T10:04:46
</commit_message>
<xml_diff>
--- a/data/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/data/BASE_CATEGORIA_PESSOAL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E323"/>
+  <dimension ref="A1:E335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7156,7 +7156,7 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="294">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -7179,7 +7179,7 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>158</v>
+        <v>3781</v>
       </c>
     </row>
     <row r="295">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7202,7 +7202,7 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>56</v>
+        <v>107</v>
       </c>
     </row>
     <row r="296">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7225,7 +7225,7 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>38</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="297">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7244,11 +7244,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>1</v>
+        <v>8398</v>
       </c>
     </row>
     <row r="298">
@@ -7257,21 +7257,21 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>273</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="299">
@@ -7280,21 +7280,21 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>7</v>
+        <v>6858</v>
       </c>
     </row>
     <row r="300">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7313,11 +7313,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="301">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7336,11 +7336,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>22</v>
+        <v>158</v>
       </c>
     </row>
     <row r="302">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7359,11 +7359,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="303">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7382,11 +7382,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>282</v>
+        <v>38</v>
       </c>
     </row>
     <row r="304">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7405,11 +7405,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>205</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
@@ -7418,7 +7418,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>53</v>
+        <v>273</v>
       </c>
     </row>
     <row r="306">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7455,7 +7455,7 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="307">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7478,7 +7478,7 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="308">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7497,11 +7497,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="309">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7520,11 +7520,11 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="310">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7543,11 +7543,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>1</v>
+        <v>282</v>
       </c>
     </row>
     <row r="311">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7566,11 +7566,11 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>24</v>
+        <v>205</v>
       </c>
     </row>
     <row r="312">
@@ -7579,21 +7579,21 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>16</v>
+        <v>53</v>
       </c>
     </row>
     <row r="313">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7612,11 +7612,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="314">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7635,11 +7635,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="315">
@@ -7648,21 +7648,21 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="316">
@@ -7671,21 +7671,21 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>1703</v>
+        <v>17</v>
       </c>
     </row>
     <row r="317">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="318">
@@ -7717,7 +7717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7731,7 +7731,7 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>4125</v>
+        <v>24</v>
       </c>
     </row>
     <row r="319">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -7754,7 +7754,7 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>21486</v>
+        <v>16</v>
       </c>
     </row>
     <row r="320">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -7777,7 +7777,7 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>14673</v>
+        <v>32</v>
       </c>
     </row>
     <row r="321">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -7796,11 +7796,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>155811</v>
+        <v>40</v>
       </c>
     </row>
     <row r="322">
@@ -7809,21 +7809,21 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>39906</v>
+        <v>32</v>
       </c>
     </row>
     <row r="323">
@@ -7832,20 +7832,296 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
+          <t>1941 - EGE-SEPLAG</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
           <t>1261 - SEE</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr">
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
         <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E323" t="n">
+      <c r="E335" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>